<commit_message>
Stram inn mobilvisning og rydde noter
</commit_message>
<xml_diff>
--- a/data/arbeidsfiler/weekly_results_2026.xlsx
+++ b/data/arbeidsfiler/weekly_results_2026.xlsx
@@ -26291,11 +26291,7 @@
       <c r="N253" t="n">
         <v>5</v>
       </c>
-      <c r="O253" t="inlineStr">
-        <is>
-          <t>Netto 16:05</t>
-        </is>
-      </c>
+      <c r="O253" t="inlineStr"/>
       <c r="P253" t="inlineStr">
         <is>
           <t>Fredrikstadløpet 5 km manuell registrering fra bilde</t>
@@ -26388,11 +26384,7 @@
       <c r="N254" t="n">
         <v>56</v>
       </c>
-      <c r="O254" t="inlineStr">
-        <is>
-          <t>Netto 20:55</t>
-        </is>
-      </c>
+      <c r="O254" t="inlineStr"/>
       <c r="P254" t="inlineStr">
         <is>
           <t>Fredrikstadløpet 5 km manuell registrering fra bilde</t>
@@ -26485,11 +26477,7 @@
       <c r="N255" t="n">
         <v>116</v>
       </c>
-      <c r="O255" t="inlineStr">
-        <is>
-          <t>Netto 25:25</t>
-        </is>
-      </c>
+      <c r="O255" t="inlineStr"/>
       <c r="P255" t="inlineStr">
         <is>
           <t>Fredrikstadløpet 5 km manuell registrering fra bilde</t>
@@ -26580,11 +26568,7 @@
       <c r="L256" t="inlineStr"/>
       <c r="M256" t="inlineStr"/>
       <c r="N256" t="inlineStr"/>
-      <c r="O256" t="inlineStr">
-        <is>
-          <t>Manuell registrering fra tekst. BIB 14445. NC.</t>
-        </is>
-      </c>
+      <c r="O256" t="inlineStr"/>
       <c r="P256" t="inlineStr">
         <is>
           <t>Milano Marathon manuell registrering fra tekst</t>

</xml_diff>

<commit_message>
Oppdater resultatdata med ny Milano-rad
</commit_message>
<xml_diff>
--- a/data/arbeidsfiler/weekly_results_2026.xlsx
+++ b/data/arbeidsfiler/weekly_results_2026.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE379"/>
+  <dimension ref="A1:AE381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40886,10 +40886,8 @@
       </c>
       <c r="L379" t="inlineStr"/>
       <c r="M379" t="inlineStr"/>
-      <c r="N379" t="inlineStr">
-        <is>
-          <t>13054</t>
-        </is>
+      <c r="N379" t="n">
+        <v>13054</v>
       </c>
       <c r="O379" t="inlineStr">
         <is>
@@ -40928,10 +40926,8 @@
           <t>M2F</t>
         </is>
       </c>
-      <c r="Z379" t="inlineStr">
-        <is>
-          <t>132</t>
-        </is>
+      <c r="Z379" t="n">
+        <v>132</v>
       </c>
       <c r="AA379" t="inlineStr"/>
       <c r="AB379" t="inlineStr"/>
@@ -40942,6 +40938,206 @@
         </is>
       </c>
       <c r="AE379" t="inlineStr">
+        <is>
+          <t>Maraton</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B380" t="n">
+        <v>15</v>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Cherry Blossom 10 Mile</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>10 mile</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>M40-44</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Bj?rnar Slettv?g</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr"/>
+      <c r="H380" t="inlineStr"/>
+      <c r="I380" t="inlineStr"/>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>55:32</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>55:32</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr"/>
+      <c r="M380" t="inlineStr"/>
+      <c r="N380" t="n">
+        <v>172</v>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>Klasseplass 8. M-rangering 144. BIB 281.</t>
+        </is>
+      </c>
+      <c r="P380" t="inlineStr">
+        <is>
+          <t>Cherry Blossom 10 Mile manuell registrering fra bilde</t>
+        </is>
+      </c>
+      <c r="Q380" t="inlineStr">
+        <is>
+          <t>manual-2026-04-12-cherry-blossom-10-mile</t>
+        </is>
+      </c>
+      <c r="R380" t="n">
+        <v>172</v>
+      </c>
+      <c r="S380" t="inlineStr"/>
+      <c r="T380" t="inlineStr"/>
+      <c r="U380" t="inlineStr"/>
+      <c r="V380" t="inlineStr">
+        <is>
+          <t>Manuell registrering</t>
+        </is>
+      </c>
+      <c r="W380" t="inlineStr"/>
+      <c r="X380" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y380" t="inlineStr">
+        <is>
+          <t>M40-44</t>
+        </is>
+      </c>
+      <c r="Z380" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA380" t="inlineStr"/>
+      <c r="AB380" t="inlineStr"/>
+      <c r="AC380" t="inlineStr"/>
+      <c r="AD380" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE380" t="inlineStr">
+        <is>
+          <t>10 mile</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B381" t="n">
+        <v>15</v>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Milano Marathon</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Maraton</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Martin Stray Egeberg</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr"/>
+      <c r="H381" t="inlineStr"/>
+      <c r="I381" t="inlineStr"/>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>2:32:43</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>2:32:43</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr"/>
+      <c r="M381" t="inlineStr"/>
+      <c r="N381" t="inlineStr"/>
+      <c r="O381" t="inlineStr">
+        <is>
+          <t>Manuell registrering fra tekst. BIB 11436. NC.</t>
+        </is>
+      </c>
+      <c r="P381" t="inlineStr">
+        <is>
+          <t>Milano Marathon manuell registrering fra tekst</t>
+        </is>
+      </c>
+      <c r="Q381" t="inlineStr">
+        <is>
+          <t>manual-2026-04-12-milano-marathon-martin</t>
+        </is>
+      </c>
+      <c r="R381" t="inlineStr"/>
+      <c r="S381" t="inlineStr"/>
+      <c r="T381" t="inlineStr"/>
+      <c r="U381" t="inlineStr"/>
+      <c r="V381" t="inlineStr">
+        <is>
+          <t>Manuell registrering</t>
+        </is>
+      </c>
+      <c r="W381" t="inlineStr"/>
+      <c r="X381" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y381" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="Z381" t="inlineStr"/>
+      <c r="AA381" t="inlineStr">
+        <is>
+          <t>1:15:16</t>
+        </is>
+      </c>
+      <c r="AB381" t="inlineStr"/>
+      <c r="AC381" t="inlineStr"/>
+      <c r="AD381" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE381" t="inlineStr">
         <is>
           <t>Maraton</t>
         </is>

</xml_diff>

<commit_message>
Samle Holmestrand maraton under ett løpsnavn
</commit_message>
<xml_diff>
--- a/data/arbeidsfiler/weekly_results_2026.xlsx
+++ b/data/arbeidsfiler/weekly_results_2026.xlsx
@@ -26164,7 +26164,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Holmestrand maraton 5k</t>
+          <t>Holmestrand maraton</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -26203,7 +26203,7 @@
       <c r="O252" t="inlineStr"/>
       <c r="P252" t="inlineStr">
         <is>
-          <t>Holmestrand maraton 5k uke 15 manuell registrering</t>
+          <t>Holmestrand maraton uke 15 manuell registrering</t>
         </is>
       </c>
       <c r="Q252" t="inlineStr">

</xml_diff>

<commit_message>
Fjern database-lenke fra nettsiden
</commit_message>
<xml_diff>
--- a/data/arbeidsfiler/weekly_results_2026.xlsx
+++ b/data/arbeidsfiler/weekly_results_2026.xlsx
@@ -27409,12 +27409,12 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="M264" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="N264" t="n">
@@ -27466,19 +27466,11 @@
       </c>
       <c r="AA264" t="inlineStr">
         <is>
-          <t>19:28</t>
-        </is>
-      </c>
-      <c r="AB264" t="inlineStr">
-        <is>
-          <t>11:32</t>
-        </is>
-      </c>
-      <c r="AC264" t="inlineStr">
-        <is>
-          <t>-7:56</t>
-        </is>
-      </c>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="AB264" t="inlineStr"/>
+      <c r="AC264" t="inlineStr"/>
       <c r="AD264" t="inlineStr"/>
       <c r="AE264" t="inlineStr"/>
     </row>
@@ -42383,10 +42375,8 @@
           <t>19:28</t>
         </is>
       </c>
-      <c r="N392" t="inlineStr">
-        <is>
-          <t>1180</t>
-        </is>
+      <c r="N392" t="n">
+        <v>1180</v>
       </c>
       <c r="O392" t="inlineStr"/>
       <c r="P392" t="inlineStr">
@@ -42421,10 +42411,8 @@
           <t>M23-34</t>
         </is>
       </c>
-      <c r="Z392" t="inlineStr">
-        <is>
-          <t>568</t>
-        </is>
+      <c r="Z392" t="n">
+        <v>568</v>
       </c>
       <c r="AA392" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Import Bislett r4 results
</commit_message>
<xml_diff>
--- a/data/arbeidsfiler/weekly_results_2026.xlsx
+++ b/data/arbeidsfiler/weekly_results_2026.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE392"/>
+  <dimension ref="A1:AE404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28345,10 +28345,8 @@
           <t>16:18</t>
         </is>
       </c>
-      <c r="N272" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="N272" t="n">
+        <v>3</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -30919,10 +30917,8 @@
           <t>16:55</t>
         </is>
       </c>
-      <c r="N294" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="N294" t="n">
+        <v>13</v>
       </c>
       <c r="O294" t="inlineStr"/>
       <c r="P294" t="inlineStr">
@@ -31155,10 +31151,8 @@
           <t>17:19</t>
         </is>
       </c>
-      <c r="N296" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="N296" t="n">
+        <v>16</v>
       </c>
       <c r="O296" t="inlineStr"/>
       <c r="P296" t="inlineStr">
@@ -31274,10 +31268,8 @@
           <t>17:22</t>
         </is>
       </c>
-      <c r="N297" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
+      <c r="N297" t="n">
+        <v>17</v>
       </c>
       <c r="O297" t="inlineStr"/>
       <c r="P297" t="inlineStr">
@@ -31510,10 +31502,8 @@
           <t>16:37</t>
         </is>
       </c>
-      <c r="N299" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
+      <c r="N299" t="n">
+        <v>19</v>
       </c>
       <c r="O299" t="inlineStr"/>
       <c r="P299" t="inlineStr">
@@ -31980,10 +31970,8 @@
           <t>17:22</t>
         </is>
       </c>
-      <c r="N303" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
+      <c r="N303" t="n">
+        <v>22</v>
       </c>
       <c r="O303" t="inlineStr"/>
       <c r="P303" t="inlineStr">
@@ -32099,10 +32087,8 @@
           <t>17:22</t>
         </is>
       </c>
-      <c r="N304" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
+      <c r="N304" t="n">
+        <v>23</v>
       </c>
       <c r="O304" t="inlineStr"/>
       <c r="P304" t="inlineStr">
@@ -32803,10 +32789,8 @@
           <t>17:58</t>
         </is>
       </c>
-      <c r="N310" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="N310" t="n">
+        <v>31</v>
       </c>
       <c r="O310" t="inlineStr"/>
       <c r="P310" t="inlineStr">
@@ -33858,10 +33842,8 @@
           <t>18:40</t>
         </is>
       </c>
-      <c r="N319" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="N319" t="n">
+        <v>45</v>
       </c>
       <c r="O319" t="inlineStr"/>
       <c r="P319" t="inlineStr">
@@ -35028,10 +35010,8 @@
           <t>19:10</t>
         </is>
       </c>
-      <c r="N329" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
+      <c r="N329" t="n">
+        <v>65</v>
       </c>
       <c r="O329" t="inlineStr"/>
       <c r="P329" t="inlineStr">
@@ -35147,10 +35127,8 @@
           <t>19:11</t>
         </is>
       </c>
-      <c r="N330" t="inlineStr">
-        <is>
-          <t>66</t>
-        </is>
+      <c r="N330" t="n">
+        <v>66</v>
       </c>
       <c r="O330" t="inlineStr"/>
       <c r="P330" t="inlineStr">
@@ -35266,10 +35244,8 @@
           <t>18:53</t>
         </is>
       </c>
-      <c r="N331" t="inlineStr">
-        <is>
-          <t>73</t>
-        </is>
+      <c r="N331" t="n">
+        <v>73</v>
       </c>
       <c r="O331" t="inlineStr"/>
       <c r="P331" t="inlineStr">
@@ -35502,10 +35478,8 @@
           <t>18:58</t>
         </is>
       </c>
-      <c r="N333" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
+      <c r="N333" t="n">
+        <v>80</v>
       </c>
       <c r="O333" t="inlineStr"/>
       <c r="P333" t="inlineStr">
@@ -35621,10 +35595,8 @@
           <t>19:09</t>
         </is>
       </c>
-      <c r="N334" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
+      <c r="N334" t="n">
+        <v>83</v>
       </c>
       <c r="O334" t="inlineStr"/>
       <c r="P334" t="inlineStr">
@@ -36091,10 +36063,8 @@
           <t>19:36</t>
         </is>
       </c>
-      <c r="N338" t="inlineStr">
-        <is>
-          <t>92</t>
-        </is>
+      <c r="N338" t="n">
+        <v>92</v>
       </c>
       <c r="O338" t="inlineStr"/>
       <c r="P338" t="inlineStr">
@@ -36444,10 +36414,8 @@
           <t>19:50</t>
         </is>
       </c>
-      <c r="N341" t="inlineStr">
-        <is>
-          <t>104</t>
-        </is>
+      <c r="N341" t="n">
+        <v>104</v>
       </c>
       <c r="O341" t="inlineStr"/>
       <c r="P341" t="inlineStr">
@@ -36563,10 +36531,8 @@
           <t>19:43</t>
         </is>
       </c>
-      <c r="N342" t="inlineStr">
-        <is>
-          <t>109</t>
-        </is>
+      <c r="N342" t="n">
+        <v>109</v>
       </c>
       <c r="O342" t="inlineStr"/>
       <c r="P342" t="inlineStr">
@@ -37033,10 +36999,8 @@
           <t>19:21</t>
         </is>
       </c>
-      <c r="N346" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
+      <c r="N346" t="n">
+        <v>123</v>
       </c>
       <c r="O346" t="inlineStr"/>
       <c r="P346" t="inlineStr">
@@ -37386,10 +37350,8 @@
           <t>20:02</t>
         </is>
       </c>
-      <c r="N349" t="inlineStr">
-        <is>
-          <t>131</t>
-        </is>
+      <c r="N349" t="n">
+        <v>131</v>
       </c>
       <c r="O349" t="inlineStr"/>
       <c r="P349" t="inlineStr">
@@ -37622,10 +37584,8 @@
           <t>19:50</t>
         </is>
       </c>
-      <c r="N351" t="inlineStr">
-        <is>
-          <t>137</t>
-        </is>
+      <c r="N351" t="n">
+        <v>137</v>
       </c>
       <c r="O351" t="inlineStr"/>
       <c r="P351" t="inlineStr">
@@ -37858,10 +37818,8 @@
           <t>19:57</t>
         </is>
       </c>
-      <c r="N353" t="inlineStr">
-        <is>
-          <t>143</t>
-        </is>
+      <c r="N353" t="n">
+        <v>143</v>
       </c>
       <c r="O353" t="inlineStr"/>
       <c r="P353" t="inlineStr">
@@ -38328,10 +38286,8 @@
           <t>20:31</t>
         </is>
       </c>
-      <c r="N357" t="inlineStr">
-        <is>
-          <t>173</t>
-        </is>
+      <c r="N357" t="n">
+        <v>173</v>
       </c>
       <c r="O357" t="inlineStr"/>
       <c r="P357" t="inlineStr">
@@ -38564,10 +38520,8 @@
           <t>20:38</t>
         </is>
       </c>
-      <c r="N359" t="inlineStr">
-        <is>
-          <t>190</t>
-        </is>
+      <c r="N359" t="n">
+        <v>190</v>
       </c>
       <c r="O359" t="inlineStr"/>
       <c r="P359" t="inlineStr">
@@ -38683,10 +38637,8 @@
           <t>20:44</t>
         </is>
       </c>
-      <c r="N360" t="inlineStr">
-        <is>
-          <t>192</t>
-        </is>
+      <c r="N360" t="n">
+        <v>192</v>
       </c>
       <c r="O360" t="inlineStr"/>
       <c r="P360" t="inlineStr">
@@ -38802,10 +38754,8 @@
           <t>20:51</t>
         </is>
       </c>
-      <c r="N361" t="inlineStr">
-        <is>
-          <t>201</t>
-        </is>
+      <c r="N361" t="n">
+        <v>201</v>
       </c>
       <c r="O361" t="inlineStr"/>
       <c r="P361" t="inlineStr">
@@ -38921,10 +38871,8 @@
           <t>20:58</t>
         </is>
       </c>
-      <c r="N362" t="inlineStr">
-        <is>
-          <t>207</t>
-        </is>
+      <c r="N362" t="n">
+        <v>207</v>
       </c>
       <c r="O362" t="inlineStr"/>
       <c r="P362" t="inlineStr">
@@ -39040,10 +38988,8 @@
           <t>20:34</t>
         </is>
       </c>
-      <c r="N363" t="inlineStr">
-        <is>
-          <t>225</t>
-        </is>
+      <c r="N363" t="n">
+        <v>225</v>
       </c>
       <c r="O363" t="inlineStr"/>
       <c r="P363" t="inlineStr">
@@ -39276,10 +39222,8 @@
           <t>20:54</t>
         </is>
       </c>
-      <c r="N365" t="inlineStr">
-        <is>
-          <t>235</t>
-        </is>
+      <c r="N365" t="n">
+        <v>235</v>
       </c>
       <c r="O365" t="inlineStr"/>
       <c r="P365" t="inlineStr">
@@ -39629,10 +39573,8 @@
           <t>20:37</t>
         </is>
       </c>
-      <c r="N368" t="inlineStr">
-        <is>
-          <t>259</t>
-        </is>
+      <c r="N368" t="n">
+        <v>259</v>
       </c>
       <c r="O368" t="inlineStr"/>
       <c r="P368" t="inlineStr">
@@ -39748,10 +39690,8 @@
           <t>21:07</t>
         </is>
       </c>
-      <c r="N369" t="inlineStr">
-        <is>
-          <t>261</t>
-        </is>
+      <c r="N369" t="n">
+        <v>261</v>
       </c>
       <c r="O369" t="inlineStr"/>
       <c r="P369" t="inlineStr">
@@ -39867,10 +39807,8 @@
           <t>21:17</t>
         </is>
       </c>
-      <c r="N370" t="inlineStr">
-        <is>
-          <t>294</t>
-        </is>
+      <c r="N370" t="n">
+        <v>294</v>
       </c>
       <c r="O370" t="inlineStr"/>
       <c r="P370" t="inlineStr">
@@ -40337,10 +40275,8 @@
           <t>22:35</t>
         </is>
       </c>
-      <c r="N374" t="inlineStr">
-        <is>
-          <t>388</t>
-        </is>
+      <c r="N374" t="n">
+        <v>388</v>
       </c>
       <c r="O374" t="inlineStr"/>
       <c r="P374" t="inlineStr">
@@ -40573,10 +40509,8 @@
           <t>22:20</t>
         </is>
       </c>
-      <c r="N376" t="inlineStr">
-        <is>
-          <t>459</t>
-        </is>
+      <c r="N376" t="n">
+        <v>459</v>
       </c>
       <c r="O376" t="inlineStr"/>
       <c r="P376" t="inlineStr">
@@ -40692,10 +40626,8 @@
           <t>23:23</t>
         </is>
       </c>
-      <c r="N377" t="inlineStr">
-        <is>
-          <t>461</t>
-        </is>
+      <c r="N377" t="n">
+        <v>461</v>
       </c>
       <c r="O377" t="inlineStr"/>
       <c r="P377" t="inlineStr">
@@ -41043,10 +40975,8 @@
           <t>24:16</t>
         </is>
       </c>
-      <c r="N380" t="inlineStr">
-        <is>
-          <t>574</t>
-        </is>
+      <c r="N380" t="n">
+        <v>574</v>
       </c>
       <c r="O380" t="inlineStr"/>
       <c r="P380" t="inlineStr">
@@ -41162,10 +41092,8 @@
           <t>24:18</t>
         </is>
       </c>
-      <c r="N381" t="inlineStr">
-        <is>
-          <t>596</t>
-        </is>
+      <c r="N381" t="n">
+        <v>596</v>
       </c>
       <c r="O381" t="inlineStr"/>
       <c r="P381" t="inlineStr">
@@ -41281,10 +41209,8 @@
           <t>27:43</t>
         </is>
       </c>
-      <c r="N382" t="inlineStr">
-        <is>
-          <t>976</t>
-        </is>
+      <c r="N382" t="n">
+        <v>976</v>
       </c>
       <c r="O382" t="inlineStr"/>
       <c r="P382" t="inlineStr">
@@ -41400,10 +41326,8 @@
           <t>20:08</t>
         </is>
       </c>
-      <c r="N383" t="inlineStr">
-        <is>
-          <t>271</t>
-        </is>
+      <c r="N383" t="n">
+        <v>271</v>
       </c>
       <c r="O383" t="inlineStr"/>
       <c r="P383" t="inlineStr">
@@ -42517,6 +42441,1202 @@
       <c r="AE392" t="inlineStr">
         <is>
           <t>10 km</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B393" t="n">
+        <v>16</v>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Aleksander Amundsen</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr"/>
+      <c r="H393" t="inlineStr"/>
+      <c r="I393" t="inlineStr"/>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr"/>
+      <c r="M393" t="inlineStr"/>
+      <c r="N393" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="O393" t="inlineStr"/>
+      <c r="P393" t="inlineStr">
+        <is>
+          <t>Aleksander Amundsen: 10:07</t>
+        </is>
+      </c>
+      <c r="Q393" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R393" t="n">
+        <v>1</v>
+      </c>
+      <c r="S393" t="inlineStr"/>
+      <c r="T393" t="inlineStr"/>
+      <c r="U393" t="inlineStr"/>
+      <c r="V393" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W393" t="inlineStr"/>
+      <c r="X393" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y393" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="Z393" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AA393" t="inlineStr"/>
+      <c r="AB393" t="inlineStr"/>
+      <c r="AC393" t="inlineStr"/>
+      <c r="AD393" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE393" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B394" t="n">
+        <v>16</v>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Erik Bjørgum</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr"/>
+      <c r="H394" t="inlineStr"/>
+      <c r="I394" t="inlineStr"/>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr"/>
+      <c r="M394" t="inlineStr"/>
+      <c r="N394" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="O394" t="inlineStr"/>
+      <c r="P394" t="inlineStr">
+        <is>
+          <t>Erik Bjørgum: 10:09</t>
+        </is>
+      </c>
+      <c r="Q394" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R394" t="n">
+        <v>2</v>
+      </c>
+      <c r="S394" t="inlineStr"/>
+      <c r="T394" t="inlineStr"/>
+      <c r="U394" t="inlineStr"/>
+      <c r="V394" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W394" t="inlineStr"/>
+      <c r="X394" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y394" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="Z394" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AA394" t="inlineStr"/>
+      <c r="AB394" t="inlineStr"/>
+      <c r="AC394" t="inlineStr"/>
+      <c r="AD394" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE394" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B395" t="n">
+        <v>16</v>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Thomas Nordbø Berg</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr"/>
+      <c r="H395" t="inlineStr"/>
+      <c r="I395" t="inlineStr"/>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>10:16</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>10:16</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr"/>
+      <c r="M395" t="inlineStr"/>
+      <c r="N395" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="O395" t="inlineStr"/>
+      <c r="P395" t="inlineStr">
+        <is>
+          <t>Thomas Nordbø Berg: 10:16</t>
+        </is>
+      </c>
+      <c r="Q395" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R395" t="n">
+        <v>3</v>
+      </c>
+      <c r="S395" t="inlineStr"/>
+      <c r="T395" t="inlineStr"/>
+      <c r="U395" t="inlineStr"/>
+      <c r="V395" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W395" t="inlineStr"/>
+      <c r="X395" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y395" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="Z395" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="AA395" t="inlineStr"/>
+      <c r="AB395" t="inlineStr"/>
+      <c r="AC395" t="inlineStr"/>
+      <c r="AD395" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE395" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B396" t="n">
+        <v>16</v>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Sven Thelin</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr"/>
+      <c r="H396" t="inlineStr"/>
+      <c r="I396" t="inlineStr"/>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr"/>
+      <c r="M396" t="inlineStr"/>
+      <c r="N396" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="O396" t="inlineStr"/>
+      <c r="P396" t="inlineStr">
+        <is>
+          <t>Sven Thelin: 10:25</t>
+        </is>
+      </c>
+      <c r="Q396" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R396" t="n">
+        <v>4</v>
+      </c>
+      <c r="S396" t="inlineStr"/>
+      <c r="T396" t="inlineStr"/>
+      <c r="U396" t="inlineStr"/>
+      <c r="V396" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W396" t="inlineStr"/>
+      <c r="X396" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y396" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="Z396" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="AA396" t="inlineStr"/>
+      <c r="AB396" t="inlineStr"/>
+      <c r="AC396" t="inlineStr"/>
+      <c r="AD396" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE396" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B397" t="n">
+        <v>16</v>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Erling Syversveen Lie</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr"/>
+      <c r="H397" t="inlineStr"/>
+      <c r="I397" t="inlineStr"/>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr"/>
+      <c r="M397" t="inlineStr"/>
+      <c r="N397" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="O397" t="inlineStr"/>
+      <c r="P397" t="inlineStr">
+        <is>
+          <t>Erling Syversveen Lie: 11:21</t>
+        </is>
+      </c>
+      <c r="Q397" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R397" t="n">
+        <v>5</v>
+      </c>
+      <c r="S397" t="inlineStr"/>
+      <c r="T397" t="inlineStr"/>
+      <c r="U397" t="inlineStr"/>
+      <c r="V397" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W397" t="inlineStr"/>
+      <c r="X397" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y397" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="Z397" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="AA397" t="inlineStr"/>
+      <c r="AB397" t="inlineStr"/>
+      <c r="AC397" t="inlineStr"/>
+      <c r="AD397" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE397" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B398" t="n">
+        <v>16</v>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>K ?pen</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Sissel Hegdahl Oversand</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr"/>
+      <c r="H398" t="inlineStr"/>
+      <c r="I398" t="inlineStr"/>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr"/>
+      <c r="M398" t="inlineStr"/>
+      <c r="N398" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="O398" t="inlineStr"/>
+      <c r="P398" t="inlineStr">
+        <is>
+          <t>Sissel Hegdahl Oversand: 11:55</t>
+        </is>
+      </c>
+      <c r="Q398" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R398" t="n">
+        <v>6</v>
+      </c>
+      <c r="S398" t="inlineStr"/>
+      <c r="T398" t="inlineStr"/>
+      <c r="U398" t="inlineStr"/>
+      <c r="V398" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W398" t="inlineStr"/>
+      <c r="X398" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="Y398" t="inlineStr">
+        <is>
+          <t>K ?pen</t>
+        </is>
+      </c>
+      <c r="Z398" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA398" t="inlineStr"/>
+      <c r="AB398" t="inlineStr"/>
+      <c r="AC398" t="inlineStr"/>
+      <c r="AD398" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="AE398" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B399" t="n">
+        <v>16</v>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>K ?pen</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Ingrid Skomedal Klovning</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr"/>
+      <c r="H399" t="inlineStr"/>
+      <c r="I399" t="inlineStr"/>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>12:11</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>12:11</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr"/>
+      <c r="M399" t="inlineStr"/>
+      <c r="N399" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O399" t="inlineStr"/>
+      <c r="P399" t="inlineStr">
+        <is>
+          <t>Ingrid Skomedal Klovning: 12:11</t>
+        </is>
+      </c>
+      <c r="Q399" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R399" t="n">
+        <v>7</v>
+      </c>
+      <c r="S399" t="inlineStr"/>
+      <c r="T399" t="inlineStr"/>
+      <c r="U399" t="inlineStr"/>
+      <c r="V399" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W399" t="inlineStr"/>
+      <c r="X399" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="Y399" t="inlineStr">
+        <is>
+          <t>K ?pen</t>
+        </is>
+      </c>
+      <c r="Z399" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA399" t="inlineStr"/>
+      <c r="AB399" t="inlineStr"/>
+      <c r="AC399" t="inlineStr"/>
+      <c r="AD399" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="AE399" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B400" t="n">
+        <v>16</v>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Sigurd Skomedal Klovning</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr"/>
+      <c r="H400" t="inlineStr"/>
+      <c r="I400" t="inlineStr"/>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>12:12</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>12:12</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr"/>
+      <c r="M400" t="inlineStr"/>
+      <c r="N400" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="O400" t="inlineStr"/>
+      <c r="P400" t="inlineStr">
+        <is>
+          <t>Sigurd Skomedal Klovning: 12:12</t>
+        </is>
+      </c>
+      <c r="Q400" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R400" t="n">
+        <v>8</v>
+      </c>
+      <c r="S400" t="inlineStr"/>
+      <c r="T400" t="inlineStr"/>
+      <c r="U400" t="inlineStr"/>
+      <c r="V400" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W400" t="inlineStr"/>
+      <c r="X400" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y400" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="Z400" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="AA400" t="inlineStr"/>
+      <c r="AB400" t="inlineStr"/>
+      <c r="AC400" t="inlineStr"/>
+      <c r="AD400" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE400" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B401" t="n">
+        <v>16</v>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Christian Lillebo</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr"/>
+      <c r="H401" t="inlineStr"/>
+      <c r="I401" t="inlineStr"/>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr"/>
+      <c r="M401" t="inlineStr"/>
+      <c r="N401" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="O401" t="inlineStr"/>
+      <c r="P401" t="inlineStr">
+        <is>
+          <t>Christian Lillebo: 12:25</t>
+        </is>
+      </c>
+      <c r="Q401" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R401" t="n">
+        <v>9</v>
+      </c>
+      <c r="S401" t="inlineStr"/>
+      <c r="T401" t="inlineStr"/>
+      <c r="U401" t="inlineStr"/>
+      <c r="V401" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W401" t="inlineStr"/>
+      <c r="X401" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y401" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="Z401" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="AA401" t="inlineStr"/>
+      <c r="AB401" t="inlineStr"/>
+      <c r="AC401" t="inlineStr"/>
+      <c r="AD401" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE401" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B402" t="n">
+        <v>16</v>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Sveinung Nersten</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr"/>
+      <c r="H402" t="inlineStr"/>
+      <c r="I402" t="inlineStr"/>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr"/>
+      <c r="M402" t="inlineStr"/>
+      <c r="N402" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="O402" t="inlineStr"/>
+      <c r="P402" t="inlineStr">
+        <is>
+          <t>Sveinung Nersten: 12:39</t>
+        </is>
+      </c>
+      <c r="Q402" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R402" t="n">
+        <v>10</v>
+      </c>
+      <c r="S402" t="inlineStr"/>
+      <c r="T402" t="inlineStr"/>
+      <c r="U402" t="inlineStr"/>
+      <c r="V402" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W402" t="inlineStr"/>
+      <c r="X402" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y402" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="Z402" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="AA402" t="inlineStr"/>
+      <c r="AB402" t="inlineStr"/>
+      <c r="AC402" t="inlineStr"/>
+      <c r="AD402" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE402" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B403" t="n">
+        <v>16</v>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Fredrik Camilo Halsbog</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr"/>
+      <c r="H403" t="inlineStr"/>
+      <c r="I403" t="inlineStr"/>
+      <c r="J403" t="inlineStr"/>
+      <c r="K403" t="inlineStr"/>
+      <c r="L403" t="inlineStr"/>
+      <c r="M403" t="inlineStr"/>
+      <c r="N403" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="O403" t="inlineStr"/>
+      <c r="P403" t="inlineStr">
+        <is>
+          <t>Fredrik Camilo Halsbog: DNF</t>
+        </is>
+      </c>
+      <c r="Q403" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R403" t="n">
+        <v>11</v>
+      </c>
+      <c r="S403" t="inlineStr"/>
+      <c r="T403" t="inlineStr"/>
+      <c r="U403" t="inlineStr"/>
+      <c r="V403" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W403" t="inlineStr"/>
+      <c r="X403" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y403" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="Z403" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AA403" t="inlineStr"/>
+      <c r="AB403" t="inlineStr"/>
+      <c r="AC403" t="inlineStr"/>
+      <c r="AD403" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE403" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B404" t="n">
+        <v>16</v>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Bislett distanseserie 4- 3K</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>3000 m</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Kristian Frøyen</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr"/>
+      <c r="H404" t="inlineStr"/>
+      <c r="I404" t="inlineStr"/>
+      <c r="J404" t="inlineStr"/>
+      <c r="K404" t="inlineStr"/>
+      <c r="L404" t="inlineStr"/>
+      <c r="M404" t="inlineStr"/>
+      <c r="N404" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="O404" t="inlineStr"/>
+      <c r="P404" t="inlineStr">
+        <is>
+          <t>Kristian Frøyen: DNF</t>
+        </is>
+      </c>
+      <c r="Q404" t="inlineStr">
+        <is>
+          <t>racedays-bislett-s2r4-2026-04-19</t>
+        </is>
+      </c>
+      <c r="R404" t="n">
+        <v>12</v>
+      </c>
+      <c r="S404" t="inlineStr"/>
+      <c r="T404" t="inlineStr"/>
+      <c r="U404" t="inlineStr"/>
+      <c r="V404" t="inlineStr">
+        <is>
+          <t>Bislett Racedays CSV import</t>
+        </is>
+      </c>
+      <c r="W404" t="inlineStr"/>
+      <c r="X404" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Y404" t="inlineStr">
+        <is>
+          <t>M ?pen</t>
+        </is>
+      </c>
+      <c r="Z404" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AA404" t="inlineStr"/>
+      <c r="AB404" t="inlineStr"/>
+      <c r="AC404" t="inlineStr"/>
+      <c r="AD404" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE404" t="inlineStr">
+        <is>
+          <t>3000 m</t>
         </is>
       </c>
     </row>

</xml_diff>